<commit_message>
rerun every stage on the reviewed methods
</commit_message>
<xml_diff>
--- a/02_HRvLR_groups/Figures/F1_Overview/c_data/f1_overview.xlsx
+++ b/02_HRvLR_groups/Figures/F1_Overview/c_data/f1_overview.xlsx
@@ -39,7 +39,7 @@
     <t>pca_proteome</t>
   </si>
   <si>
-    <t>Panel c, left: PC1 and PC2 per sample (02_Contrasts, pca).</t>
+    <t>Panel c, left: PC1 and PC2 per sample (02_DEP, pca).</t>
   </si>
   <si>
     <t>pca_phenotype</t>
@@ -51,7 +51,7 @@
     <t>permanova</t>
   </si>
   <si>
-    <t>Panel c: PERMANOVA for the proteome (time, arm) and the phenotype (time) (02_Contrasts).</t>
+    <t>Panel c: PERMANOVA for the proteome (time, arm) and the phenotype (time) (02_DEP).</t>
   </si>
   <si>
     <t>pathways</t>

</xml_diff>